<commit_message>
Update latest.xlsx 2026-10-15 16:45
</commit_message>
<xml_diff>
--- a/latest.xlsx
+++ b/latest.xlsx
@@ -1818,9 +1818,9 @@
         <t>관세 0원 : 한-EU FTA 협정세율(세율구분 FEU1 이가) 적용, HS 8414.59-9000 (신고필증 14008-26-101205M, 수리일 2026-07-27)</t>
       </text>
     </comment>
-    <comment ref="K38" authorId="0" shapeId="0">
+    <comment ref="K38" authorId="1" shapeId="0">
       <text>
-        <t>분할송금 1차: USD 50,000 (2026-09-15, 적용환율 1,364.10) = 68,205,000원. Invoice USD 807,233 중 잔여 USD 757,233 미송금 (지급합의 일정: 2026-11-15 USD 250,000 / 2026-12-31 USD 507,233). 원화환산액은 송금 완료분만 반영, 잔여분 송금 시 가산</t>
+        <t>분할송금 1차: USD 50,000 (2026-09-15, 적용환율 1,364.10) = 68,205,000원 (J열). Invoice USD 총액 중 잔여 USD 757,233 미송금 (지급합의 일정: 2026-11-15 USD 250,000 / 2026-12-31 USD 507,233, 696-4/-5 합산). 2026-10-15 기준 잔여분은 수입신고일 신고환율(Q열)로 환산해 원가 반영 (입고 기준 취득원가, 송금 여부 무관). 잔금 송금 시 송금환율로 갱신하고 차액은 외환차손익.</t>
       </text>
     </comment>
     <comment ref="S40" authorId="0" shapeId="0">
@@ -1837,9 +1837,9 @@
 원산지: 우크라이나(UA-A)</t>
       </text>
     </comment>
-    <comment ref="K42" authorId="0" shapeId="0">
+    <comment ref="K42" authorId="1" shapeId="0">
       <text>
-        <t>분할송금 1차: USD 50,000 (2026-09-15, 적용환율 1,364.10) = 68,205,000원. Invoice USD 346,792 중 잔여 USD 296,792 미송금 (지급합의 일정: 2026-11-15 USD 100,000 / 2026-12-31 USD 196,792). 원화환산액은 송금 완료분만 반영, 잔여분 송금 시 가산</t>
+        <t>분할송금 1차: USD 50,000 (2026-09-15, 적용환율 1,364.10) = 68,205,000원 (J열). Invoice USD 총액 중 잔여 USD 296,792 미송금 (지급합의 일정: 2026-11-15 USD 250,000 / 2026-12-31 USD 507,233, 696-4/-5 합산). 2026-10-15 기준 잔여분은 수입신고일 신고환율(Q열)로 환산해 원가 반영 (입고 기준 취득원가, 송금 여부 무관). 잔금 송금 시 송금환율로 갱신하고 차액은 외환차손익.</t>
       </text>
     </comment>
     <comment ref="S43" authorId="0" shapeId="0">
@@ -2259,7 +2259,7 @@
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="241" t="inlineStr">
         <is>
-          <t>회계처리용 통합 데이터  |  기준일: 2026-10-13  |  노란색=미확인  |  보라색=라이센스/워런티  |  날짜→해당항목 좌측 배치</t>
+          <t>회계처리용 통합 데이터  |  기준일: 2026-10-15  |  노란색=미확인  |  보라색=라이센스/워런티  |  날짜→해당항목 좌측 배치</t>
         </is>
       </c>
       <c r="B2" s="219" t="n"/>
@@ -3057,7 +3057,7 @@
         <v>0</v>
       </c>
       <c r="K9" s="159">
-        <f>IFERROR(ROUND(H9*I9,0),0)</f>
+        <f>IFERROR(IF(I9&gt;0,ROUND(H9*I9,0),IF(ISNUMBER(Q9),ROUND(H9*Q9,0),0)),0)</f>
         <v/>
       </c>
       <c r="L9" s="159">
@@ -4801,7 +4801,7 @@
         <v>0</v>
       </c>
       <c r="K23" s="159">
-        <f>IFERROR(ROUND(H23*I23,0),0)</f>
+        <f>IFERROR(IF(I23&gt;0,ROUND(H23*I23,0),IF(ISNUMBER(Q23),ROUND(H23*Q23,0),0)),0)</f>
         <v/>
       </c>
       <c r="L23" s="159">
@@ -6549,8 +6549,9 @@
       <c r="J38" s="159" t="n">
         <v>68205000</v>
       </c>
-      <c r="K38" s="159" t="n">
-        <v>68205000</v>
+      <c r="K38" s="159">
+        <f>J38+ROUND((H38-IFERROR(VLOOKUP(B38,RemitTable2,4,FALSE),0))*Q38,0)</f>
+        <v/>
       </c>
       <c r="L38" s="159" t="n">
         <v>1584</v>
@@ -7013,8 +7014,9 @@
       <c r="J42" s="159" t="n">
         <v>68205000</v>
       </c>
-      <c r="K42" s="159" t="n">
-        <v>68205000</v>
+      <c r="K42" s="159">
+        <f>J42+ROUND((H42-IFERROR(VLOOKUP(B42,RemitTable2,4,FALSE),0))*Q42,0)</f>
+        <v/>
       </c>
       <c r="L42" s="159" t="n">
         <v>1584</v>
@@ -7241,20 +7243,24 @@
       <c r="H44" s="151" t="n">
         <v>14730</v>
       </c>
-      <c r="I44" s="248" t="n">
-        <v>0</v>
+      <c r="I44" s="248">
+        <f>IFERROR(VLOOKUP(B44,RemitTable2,7,FALSE),0)</f>
+        <v/>
       </c>
       <c r="J44" s="159" t="n">
         <v>0</v>
       </c>
-      <c r="K44" s="159" t="n">
-        <v>0</v>
-      </c>
-      <c r="L44" s="159" t="n">
-        <v>0</v>
-      </c>
-      <c r="M44" s="159" t="n">
-        <v>0</v>
+      <c r="K44" s="159">
+        <f>IFERROR(IF(I44&gt;0,ROUND(H44*I44,0),IF(ISNUMBER(Q44),ROUND(H44*Q44,0),0)),0)</f>
+        <v/>
+      </c>
+      <c r="L44" s="159">
+        <f>IFERROR(VLOOKUP(B44,RemitTable2,10,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="M44" s="159">
+        <f>IFERROR(VLOOKUP(B44,RemitTable2,11,FALSE),0)</f>
+        <v/>
       </c>
       <c r="N44" s="152" t="inlineStr">
         <is>
@@ -8096,7 +8102,7 @@
         <v>0</v>
       </c>
       <c r="K51" s="159">
-        <f>IFERROR(ROUND(H51*I51,0),0)</f>
+        <f>IFERROR(IF(I51&gt;0,ROUND(H51*I51,0),IF(ISNUMBER(Q51),ROUND(H51*Q51,0),0)),0)</f>
         <v/>
       </c>
       <c r="L51" s="159">
@@ -8842,7 +8848,7 @@
         <v>0</v>
       </c>
       <c r="K57" s="159">
-        <f>IFERROR(ROUND(H57*I57,0),0)</f>
+        <f>IFERROR(IF(I57&gt;0,ROUND(H57*I57,0),IF(ISNUMBER(Q57),ROUND(H57*Q57,0),0)),0)</f>
         <v/>
       </c>
       <c r="L57" s="159">
@@ -9697,7 +9703,7 @@
         <v>0</v>
       </c>
       <c r="K64" s="363">
-        <f>IFERROR(ROUND(H64*I64,0),0)</f>
+        <f>IFERROR(IF(I64&gt;0,ROUND(H64*I64,0),IF(ISNUMBER(Q64),ROUND(H64*Q64,0),0)),0)</f>
         <v/>
       </c>
       <c r="L64" s="363">
@@ -9945,7 +9951,7 @@
         <v>0</v>
       </c>
       <c r="K66" s="363">
-        <f>IFERROR(ROUND(H66*I66,0),0)</f>
+        <f>IFERROR(IF(I66&gt;0,ROUND(H66*I66,0),IF(ISNUMBER(Q66),ROUND(H66*Q66,0),0)),0)</f>
         <v/>
       </c>
       <c r="L66" s="363">
@@ -11262,7 +11268,7 @@
         <v>0</v>
       </c>
       <c r="K77" s="370">
-        <f>IFERROR(ROUND(H77*I77,0),0)</f>
+        <f>IFERROR(IF(I77&gt;0,ROUND(H77*I77,0),IF(ISNUMBER(Q77),ROUND(H77*Q77,0),0)),0)</f>
         <v/>
       </c>
       <c r="L77" s="370">
@@ -11942,20 +11948,24 @@
       <c r="H83" s="361" t="n">
         <v>450</v>
       </c>
-      <c r="I83" s="362" t="n">
-        <v>0</v>
+      <c r="I83" s="362">
+        <f>IFERROR(VLOOKUP(B83,RemitTable2,7,FALSE),0)</f>
+        <v/>
       </c>
       <c r="J83" s="363" t="n">
         <v>0</v>
       </c>
-      <c r="K83" s="363" t="n">
-        <v>0</v>
-      </c>
-      <c r="L83" s="363" t="n">
-        <v>0</v>
-      </c>
-      <c r="M83" s="363" t="n">
-        <v>0</v>
+      <c r="K83" s="363">
+        <f>IFERROR(IF(I83&gt;0,ROUND(H83*I83,0),IF(ISNUMBER(Q83),ROUND(H83*Q83,0),0)),0)</f>
+        <v/>
+      </c>
+      <c r="L83" s="363">
+        <f>IFERROR(VLOOKUP(B83,RemitTable2,10,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="M83" s="363">
+        <f>IFERROR(VLOOKUP(B83,RemitTable2,11,FALSE),0)</f>
+        <v/>
       </c>
       <c r="N83" s="357" t="inlineStr">
         <is>
@@ -12057,20 +12067,24 @@
       <c r="H84" s="361" t="n">
         <v>7407.81</v>
       </c>
-      <c r="I84" s="362" t="n">
-        <v>0</v>
+      <c r="I84" s="362">
+        <f>IFERROR(VLOOKUP(B84,RemitTable2,7,FALSE),0)</f>
+        <v/>
       </c>
       <c r="J84" s="363" t="n">
         <v>0</v>
       </c>
-      <c r="K84" s="363" t="n">
-        <v>0</v>
-      </c>
-      <c r="L84" s="363" t="n">
-        <v>0</v>
-      </c>
-      <c r="M84" s="363" t="n">
-        <v>0</v>
+      <c r="K84" s="363">
+        <f>IFERROR(IF(I84&gt;0,ROUND(H84*I84,0),IF(ISNUMBER(Q84),ROUND(H84*Q84,0),0)),0)</f>
+        <v/>
+      </c>
+      <c r="L84" s="363">
+        <f>IFERROR(VLOOKUP(B84,RemitTable2,10,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="M84" s="363">
+        <f>IFERROR(VLOOKUP(B84,RemitTable2,11,FALSE),0)</f>
+        <v/>
       </c>
       <c r="N84" s="357" t="inlineStr">
         <is>
@@ -12172,20 +12186,24 @@
       <c r="H85" s="361" t="n">
         <v>3320</v>
       </c>
-      <c r="I85" s="362" t="n">
-        <v>0</v>
+      <c r="I85" s="362">
+        <f>IFERROR(VLOOKUP(B85,RemitTable2,7,FALSE),0)</f>
+        <v/>
       </c>
       <c r="J85" s="363" t="n">
         <v>0</v>
       </c>
-      <c r="K85" s="363" t="n">
-        <v>0</v>
-      </c>
-      <c r="L85" s="363" t="n">
-        <v>0</v>
-      </c>
-      <c r="M85" s="363" t="n">
-        <v>0</v>
+      <c r="K85" s="363">
+        <f>IFERROR(IF(I85&gt;0,ROUND(H85*I85,0),IF(ISNUMBER(Q85),ROUND(H85*Q85,0),0)),0)</f>
+        <v/>
+      </c>
+      <c r="L85" s="363">
+        <f>IFERROR(VLOOKUP(B85,RemitTable2,10,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="M85" s="363">
+        <f>IFERROR(VLOOKUP(B85,RemitTable2,11,FALSE),0)</f>
+        <v/>
       </c>
       <c r="N85" s="357" t="inlineStr">
         <is>
@@ -12297,7 +12315,7 @@
         <v>0</v>
       </c>
       <c r="K86" s="363">
-        <f>IFERROR(ROUND(H86*I86,0),0)</f>
+        <f>IFERROR(IF(I86&gt;0,ROUND(H86*I86,0),IF(ISNUMBER(Q86),ROUND(H86*Q86,0),0)),0)</f>
         <v/>
       </c>
       <c r="L86" s="363">
@@ -12549,7 +12567,7 @@
         <v>0</v>
       </c>
       <c r="K88" s="363">
-        <f>IFERROR(ROUND(H88*I88,0),0)</f>
+        <f>IFERROR(IF(I88&gt;0,ROUND(H88*I88,0),IF(ISNUMBER(Q88),ROUND(H88*Q88,0),0)),0)</f>
         <v/>
       </c>
       <c r="L88" s="363">
@@ -12670,7 +12688,7 @@
         <v>0</v>
       </c>
       <c r="K89" s="363">
-        <f>IFERROR(ROUND(H89*I89,0),0)</f>
+        <f>IFERROR(IF(I89&gt;0,ROUND(H89*I89,0),IF(ISNUMBER(Q89),ROUND(H89*Q89,0),0)),0)</f>
         <v/>
       </c>
       <c r="L89" s="363">
@@ -12791,7 +12809,7 @@
         <v>0</v>
       </c>
       <c r="K90" s="363">
-        <f>IFERROR(ROUND(H90*I90,0),0)</f>
+        <f>IFERROR(IF(I90&gt;0,ROUND(H90*I90,0),IF(ISNUMBER(Q90),ROUND(H90*Q90,0),0)),0)</f>
         <v/>
       </c>
       <c r="L90" s="363">
@@ -12912,7 +12930,7 @@
         <v>0</v>
       </c>
       <c r="K91" s="363">
-        <f>IFERROR(ROUND(H91*I91,0),0)</f>
+        <f>IFERROR(IF(I91&gt;0,ROUND(H91*I91,0),IF(ISNUMBER(Q91),ROUND(H91*Q91,0),0)),0)</f>
         <v/>
       </c>
       <c r="L91" s="363">
@@ -13033,7 +13051,7 @@
         <v>0</v>
       </c>
       <c r="K92" s="363">
-        <f>IFERROR(ROUND(H92*I92,0),0)</f>
+        <f>IFERROR(IF(I92&gt;0,ROUND(H92*I92,0),IF(ISNUMBER(Q92),ROUND(H92*Q92,0),0)),0)</f>
         <v/>
       </c>
       <c r="L92" s="363">
@@ -13154,7 +13172,7 @@
         <v>0</v>
       </c>
       <c r="K93" s="363">
-        <f>IFERROR(ROUND(H93*I93,0),0)</f>
+        <f>IFERROR(IF(I93&gt;0,ROUND(H93*I93,0),IF(ISNUMBER(Q93),ROUND(H93*Q93,0),0)),0)</f>
         <v/>
       </c>
       <c r="L93" s="363">
@@ -13275,7 +13293,7 @@
         <v>0</v>
       </c>
       <c r="K94" s="363">
-        <f>IFERROR(ROUND(H94*I94,0),0)</f>
+        <f>IFERROR(IF(I94&gt;0,ROUND(H94*I94,0),IF(ISNUMBER(Q94),ROUND(H94*Q94,0),0)),0)</f>
         <v/>
       </c>
       <c r="L94" s="363">
@@ -13394,7 +13412,7 @@
         <v>0</v>
       </c>
       <c r="K95" s="379">
-        <f>IFERROR(ROUND(H95*I95,0),0)</f>
+        <f>IFERROR(IF(I95&gt;0,ROUND(H95*I95,0),IF(ISNUMBER(Q95),ROUND(H95*Q95,0),0)),0)</f>
         <v/>
       </c>
       <c r="L95" s="379">
@@ -13986,7 +14004,7 @@
         <v>0</v>
       </c>
       <c r="K100" s="379">
-        <f>IFERROR(ROUND(H100*I100,0),0)</f>
+        <f>IFERROR(IF(I100&gt;0,ROUND(H100*I100,0),IF(ISNUMBER(Q100),ROUND(H100*Q100,0),0)),0)</f>
         <v/>
       </c>
       <c r="L100" s="379">
@@ -24726,7 +24744,7 @@
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="340" t="inlineStr">
         <is>
-          <t>기준일: 2026-10-13  |  상환 완료 건은 초록색 표시  |  상환예정일 = 신한은행 PDF 만기일 기준</t>
+          <t>기준일: 2026-10-15  |  상환 완료 건은 초록색 표시  |  상환예정일 = 신한은행 PDF 만기일 기준</t>
         </is>
       </c>
     </row>

</xml_diff>